<commit_message>
Now hysteresis loops is run only for fa experiment which are not fracture, corrected some errors in the metadata and replaced api.py in api_v2.py in backend/Makefile
</commit_message>
<xml_diff>
--- a/Data/raw/TST_Mannino_2023-10_FA/TST_2023-10_FA_metadata.xlsx
+++ b/Data/raw/TST_Mannino_2023-10_FA/TST_2023-10_FA_metadata.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oros\Desktop\dataset_upload\TST_Mannino_2023-10_FA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{082FA39C-A95F-498F-8A70-98116BDFACC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0738CC38-2113-4E86-B9D6-417D1F5F813C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="15" windowWidth="20640" windowHeight="11040" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -266,9 +266,6 @@
     <t>Hardener</t>
   </si>
   <si>
-    <t>Material</t>
-  </si>
-  <si>
     <t>Sequential number</t>
   </si>
   <si>
@@ -311,9 +308,6 @@
     <t>Material info</t>
   </si>
   <si>
-    <t>CCLab</t>
-  </si>
-  <si>
     <t>Filippo Mannino</t>
   </si>
   <si>
@@ -326,19 +320,25 @@
     <t>Type II</t>
   </si>
   <si>
-    <t>Sikadur-330, epoxy resin</t>
-  </si>
-  <si>
     <t>F2-A13-631-7</t>
   </si>
   <si>
     <t>F2-A14-574-3</t>
   </si>
   <si>
-    <t>F2-A143-574-4</t>
-  </si>
-  <si>
     <t>F2-A10-506-3</t>
+  </si>
+  <si>
+    <t>Fiber Material</t>
+  </si>
+  <si>
+    <t>Epoxy Sikadur-330</t>
+  </si>
+  <si>
+    <t>GR-MeC</t>
+  </si>
+  <si>
+    <t>F2-A13-574-4</t>
   </si>
 </sst>
 </file>
@@ -526,6 +526,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -541,35 +544,18 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <fill>
         <patternFill>
@@ -697,23 +683,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>308162</xdr:colOff>
-      <xdr:row>3</xdr:row>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>7</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>1617934</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>76487</xdr:rowOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>2407069</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>150351</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
+        <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FC0C11FC-D7EF-49B6-9CF8-E8BD18A71247}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0D7FB3E-6B8D-4685-86D1-DE69B7473980}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -729,8 +715,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="23429633" y="3585883"/>
-          <a:ext cx="6096851" cy="3391373"/>
+          <a:off x="30831118" y="2181412"/>
+          <a:ext cx="5679186" cy="2167410"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1139,55 +1125,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" s="2" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
-      <c r="L1" s="15"/>
-      <c r="M1" s="15"/>
-      <c r="N1" s="15"/>
-      <c r="O1" s="15"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="16"/>
       <c r="P1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="Q1" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="R1" s="16"/>
-      <c r="S1" s="16"/>
-      <c r="T1" s="16"/>
-      <c r="U1" s="16"/>
-      <c r="V1" s="16"/>
-      <c r="W1" s="16"/>
-      <c r="X1" s="16"/>
-      <c r="Y1" s="16"/>
-      <c r="Z1" s="16"/>
-      <c r="AA1" s="16"/>
-      <c r="AB1" s="16"/>
-      <c r="AC1" s="16"/>
-      <c r="AD1" s="16"/>
-      <c r="AE1" s="16"/>
-      <c r="AF1" s="16"/>
-      <c r="AG1" s="16"/>
-      <c r="AH1" s="16"/>
-      <c r="AI1" s="16"/>
-      <c r="AJ1" s="14" t="s">
+      <c r="Q1" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="R1" s="17"/>
+      <c r="S1" s="17"/>
+      <c r="T1" s="17"/>
+      <c r="U1" s="17"/>
+      <c r="V1" s="17"/>
+      <c r="W1" s="17"/>
+      <c r="X1" s="17"/>
+      <c r="Y1" s="17"/>
+      <c r="Z1" s="17"/>
+      <c r="AA1" s="17"/>
+      <c r="AB1" s="17"/>
+      <c r="AC1" s="17"/>
+      <c r="AD1" s="17"/>
+      <c r="AE1" s="17"/>
+      <c r="AF1" s="17"/>
+      <c r="AG1" s="17"/>
+      <c r="AH1" s="17"/>
+      <c r="AI1" s="17"/>
+      <c r="AJ1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="AK1" s="14"/>
-      <c r="AL1" s="12" t="s">
+      <c r="AK1" s="15"/>
+      <c r="AL1" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="AM1" s="13"/>
+      <c r="AM1" s="14"/>
     </row>
     <row r="2" spans="1:39" s="2" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
@@ -1248,7 +1234,7 @@
         <v>57</v>
       </c>
       <c r="T2" s="4" t="s">
-        <v>77</v>
+        <v>98</v>
       </c>
       <c r="U2" s="4" t="s">
         <v>58</v>
@@ -1310,13 +1296,13 @@
     </row>
     <row r="3" spans="1:39" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>92</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>94</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>4</v>
@@ -1338,21 +1324,21 @@
       </c>
       <c r="N3" s="6"/>
       <c r="O3" s="6"/>
-      <c r="P3" s="19" t="s">
-        <v>95</v>
+      <c r="P3" s="12" t="s">
+        <v>93</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>46</v>
       </c>
       <c r="R3" s="9" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="S3" s="7"/>
       <c r="T3" s="8"/>
       <c r="U3" s="6"/>
       <c r="V3" s="6"/>
       <c r="W3" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="X3" s="6"/>
       <c r="Y3" s="6"/>
@@ -1400,32 +1386,32 @@
     <mergeCell ref="Q1:AI1"/>
   </mergeCells>
   <conditionalFormatting sqref="E3">
-    <cfRule type="expression" dxfId="7" priority="6">
+    <cfRule type="expression" dxfId="5" priority="6">
       <formula>D3="QS"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3 M3 AL3:AM3">
-    <cfRule type="expression" dxfId="6" priority="9">
+    <cfRule type="expression" dxfId="4" priority="9">
       <formula>$D$3="FA"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3">
-    <cfRule type="expression" dxfId="5" priority="5">
+    <cfRule type="expression" dxfId="3" priority="5">
       <formula>D3="OT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3 N3">
-    <cfRule type="expression" dxfId="4" priority="3">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>G3="Other"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I3">
-    <cfRule type="expression" dxfId="3" priority="7">
+    <cfRule type="expression" dxfId="1" priority="7">
       <formula>OR(E3="fracture", F3="fracture")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S3">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>Q3="Other polymers"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1508,69 +1494,69 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="15"/>
+      <c r="B1" s="16"/>
       <c r="C1" s="18" t="s">
         <v>32</v>
       </c>
       <c r="D1" s="18"/>
       <c r="E1" s="18"/>
-      <c r="F1" s="16" t="s">
+      <c r="F1" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="14" t="s">
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="K1" s="14"/>
-      <c r="L1" s="17" t="s">
+      <c r="K1" s="15"/>
+      <c r="L1" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="M1" s="17"/>
+      <c r="M1" s="19"/>
     </row>
     <row r="2" spans="1:13" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="H2" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="K2" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="L2" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="M2" s="4" t="s">
         <v>89</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
@@ -1578,7 +1564,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C3" s="6">
         <v>2729</v>
@@ -1607,7 +1593,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C4" s="6">
         <v>54318</v>
@@ -1636,7 +1622,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C5" s="6">
         <v>99680</v>
@@ -1665,7 +1651,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C6" s="6">
         <v>241732</v>

</xml_diff>